<commit_message>
started to rewrite codes
</commit_message>
<xml_diff>
--- a/data/magyar_petered_telepulesek.xlsx
+++ b/data/magyar_petered_telepulesek.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Downloads/egyetem/TDK/magyar_petered/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/Downloads/egyetem/TDK/magyar_petered_main/magyar_petered/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71D55AD0-CE9C-B946-9B24-48F2805B3DAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56A3564C-835F-784A-9752-703F669C8868}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="15760" xr2:uid="{267B8A77-B259-1C46-AB3D-9FC0ACCE92D9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="212">
   <si>
     <t>is_magyar_petered</t>
   </si>
@@ -591,6 +591,87 @@
   </si>
   <si>
     <t>Kiskunfélegyháza</t>
+  </si>
+  <si>
+    <t>is_fideszed</t>
+  </si>
+  <si>
+    <t>is_dked</t>
+  </si>
+  <si>
+    <t>Nemesgörzsöny</t>
+  </si>
+  <si>
+    <t>Soltvadkert</t>
+  </si>
+  <si>
+    <t>Lakitelek</t>
+  </si>
+  <si>
+    <t>Dabas</t>
+  </si>
+  <si>
+    <t>Ráckeve</t>
+  </si>
+  <si>
+    <t>Tinnye</t>
+  </si>
+  <si>
+    <t>Solymár</t>
+  </si>
+  <si>
+    <t>Pomáz</t>
+  </si>
+  <si>
+    <t>Nagykökényes</t>
+  </si>
+  <si>
+    <t>Lőrinci</t>
+  </si>
+  <si>
+    <t>Geszt</t>
+  </si>
+  <si>
+    <t>Tiszaladány</t>
+  </si>
+  <si>
+    <t>Jánd</t>
+  </si>
+  <si>
+    <t>Győrszentiván</t>
+  </si>
+  <si>
+    <t>Bakonyszentlászló</t>
+  </si>
+  <si>
+    <t>Sárisáp</t>
+  </si>
+  <si>
+    <t>Lepsény</t>
+  </si>
+  <si>
+    <t>Szabadbattyán</t>
+  </si>
+  <si>
+    <t>Felsőszentiván</t>
+  </si>
+  <si>
+    <t>Bácsalmás</t>
+  </si>
+  <si>
+    <t>Csikéria</t>
+  </si>
+  <si>
+    <t>Nagykőrös</t>
+  </si>
+  <si>
+    <t>Deszk</t>
+  </si>
+  <si>
+    <t>Szeghalom</t>
+  </si>
+  <si>
+    <t>Polgár</t>
   </si>
 </sst>
 </file>
@@ -962,325 +1043,622 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2A82633-472C-7C47-96D1-FD3C4D3F9067}">
-  <dimension ref="A1:A188"/>
+  <dimension ref="A1:C188"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B1" t="s">
+        <v>185</v>
+      </c>
+      <c r="C1" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B5" t="s">
+        <v>187</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B11" t="s">
+        <v>70</v>
+      </c>
+      <c r="C11" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B16" t="s">
+        <v>48</v>
+      </c>
+      <c r="C16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
+        <v>180</v>
+      </c>
+      <c r="C17" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>188</v>
+      </c>
+      <c r="C18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B19" t="s">
+        <v>184</v>
+      </c>
+      <c r="C19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
+        <v>189</v>
+      </c>
+      <c r="C20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>176</v>
+      </c>
+      <c r="C21" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>190</v>
+      </c>
+      <c r="C22" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>191</v>
+      </c>
+      <c r="C23" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B24" t="s">
+        <v>192</v>
+      </c>
+      <c r="C24" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B25" t="s">
+        <v>193</v>
+      </c>
+      <c r="C25" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B26" t="s">
+        <v>194</v>
+      </c>
+      <c r="C26" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B27" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B28" t="s">
+        <v>98</v>
+      </c>
+      <c r="C28" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B29" t="s">
+        <v>195</v>
+      </c>
+      <c r="C29" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B30" t="s">
+        <v>196</v>
+      </c>
+      <c r="C30" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B31" t="s">
+        <v>101</v>
+      </c>
+      <c r="C31" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B32" t="s">
+        <v>104</v>
+      </c>
+      <c r="C32" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B33" t="s">
+        <v>109</v>
+      </c>
+      <c r="C33" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B34" t="s">
+        <v>114</v>
+      </c>
+      <c r="C34" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B35" t="s">
+        <v>111</v>
+      </c>
+      <c r="C35" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B36" t="s">
+        <v>122</v>
+      </c>
+      <c r="C36" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B37" t="s">
+        <v>126</v>
+      </c>
+      <c r="C37" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B38" t="s">
+        <v>130</v>
+      </c>
+      <c r="C38" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B39" t="s">
+        <v>197</v>
+      </c>
+      <c r="C39" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B40" t="s">
+        <v>136</v>
+      </c>
+      <c r="C40" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B41" t="s">
+        <v>143</v>
+      </c>
+      <c r="C41" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B42" t="s">
+        <v>146</v>
+      </c>
+      <c r="C42" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B43" t="s">
+        <v>198</v>
+      </c>
+      <c r="C43" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B44" t="s">
+        <v>199</v>
+      </c>
+      <c r="C44" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="B45" t="s">
+        <v>150</v>
+      </c>
+      <c r="C45" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="C46" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="C47" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="C48" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="C49" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="C50" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="C51" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="C52" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="C53" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="C54" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>61</v>
       </c>

</xml_diff>